<commit_message>
feat: Add RationalQuadratic kernel, Live Interactive Monte Carlo Tolerance Stress-Test, Wilcoxon Rank-Sum table, and refine model hierarchy based on committee review
</commit_message>
<xml_diff>
--- a/reports/Microrobot_Defense_Validation_Report.xlsx
+++ b/reports/Microrobot_Defense_Validation_Report.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,12 +496,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RBF</t>
+          <t>Matérn 5/2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C^inf (Vô hạn lần khả vi, giả định biến thiên siêu trơn)</t>
+          <t>C^2 (2 lần khả vi, tương thích hoàn hảo với PDE đàn hồi bậc 2 - Mô hình chủ đạo)</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -511,25 +511,25 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1764</v>
+        <v>0.1983</v>
       </c>
       <c r="G2" t="n">
-        <v>64.0915</v>
+        <v>63.2316</v>
       </c>
       <c r="H2" t="n">
-        <v>46.5611</v>
+        <v>46.2004</v>
       </c>
       <c r="I2" t="n">
-        <v>3.719</v>
+        <v>3.69</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-0.1117 ± 0.4301</t>
+          <t>0.0581 ± 0.4067</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>64.9369 ± 16.8029</t>
+          <t>60.2996 ± 18.4649</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C^1 (1 lần khả vi, cho phép biến thiên dốc)</t>
+          <t>C^1 (1 lần khả vi, mô phỏng biến thiên dốc)</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -586,12 +586,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Matérn 5/2</t>
+          <t>RationalQuadratic</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>C^2 (2 lần khả vi, tương thích hoàn hảo với PDE đàn hồi)</t>
+          <t>Hỗn hợp vô hạn các RBF đa quy mô độ dài (đa tỷ lệ)</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -601,70 +601,70 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1983</v>
+        <v>0.1756</v>
       </c>
       <c r="G4" t="n">
-        <v>63.2316</v>
+        <v>64.1203</v>
       </c>
       <c r="H4" t="n">
-        <v>46.2004</v>
+        <v>46.6213</v>
       </c>
       <c r="I4" t="n">
-        <v>3.69</v>
+        <v>3.724</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0581 ± 0.4067</t>
+          <t>0.0135 ± 0.4172</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>60.2996 ± 18.4649</t>
+          <t>61.7145 ± 18.6524</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Safety factor (SF)</t>
+          <t>Stroke (µm)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RBF</t>
+          <t>RBF (Gaussian)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>C^inf (Vô hạn lần khả vi, giả định biến thiên siêu trơn)</t>
+          <t>C^inf (Vô hạn lần khả vi, nguy cơ quá trơn làm mờ đỉnh ứng suất)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.9969</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0.007900000000000001</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2419</v>
+        <v>0.1764</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1584</v>
+        <v>64.0915</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1138</v>
+        <v>46.5611</v>
       </c>
       <c r="I5" t="n">
-        <v>5.874</v>
+        <v>3.719</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-0.8108 ± 0.9292</t>
+          <t>-0.1117 ± 0.4301</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.148 ± 0.0547</t>
+          <t>64.9369 ± 16.8029</t>
         </is>
       </c>
     </row>
@@ -676,40 +676,40 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Matérn 3/2</t>
+          <t>Matérn 5/2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>C^1 (1 lần khả vi, cho phép biến thiên dốc)</t>
+          <t>C^2 (2 lần khả vi, tương thích hoàn hảo với PDE đàn hồi bậc 2 - Mô hình chủ đạo)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.9971</v>
+        <v>0.997</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0076</v>
+        <v>0.0078</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.1749</v>
+        <v>-0.1917</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1541</v>
+        <v>0.1552</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1115</v>
+        <v>0.1122</v>
       </c>
       <c r="I6" t="n">
-        <v>5.762</v>
+        <v>5.795</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-0.7572 ± 0.8872</t>
+          <t>-0.7747 ± 0.8978</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.1463 ± 0.0541</t>
+          <t>0.147 ± 0.0544</t>
         </is>
       </c>
     </row>
@@ -721,40 +721,130 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Matérn 5/2</t>
+          <t>Matérn 3/2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>C^2 (2 lần khả vi, tương thích hoàn hảo với PDE đàn hồi)</t>
+          <t>C^1 (1 lần khả vi, mô phỏng biến thiên dốc)</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.997</v>
+        <v>0.9971</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0078</v>
+        <v>0.0076</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1917</v>
+        <v>-0.1749</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1552</v>
+        <v>0.1541</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1122</v>
+        <v>0.1115</v>
       </c>
       <c r="I7" t="n">
-        <v>5.795</v>
+        <v>5.762</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>-0.7747 ± 0.8978</t>
+          <t>-0.7572 ± 0.8872</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>0.147 ± 0.0544</t>
+          <t>0.1463 ± 0.0541</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Safety factor (SF)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RationalQuadratic</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hỗn hợp vô hạn các RBF đa quy mô độ dài (đa tỷ lệ)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0142</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.2069</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.1561</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.1123</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5.807</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>-0.7997 ± 0.9208</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.1477 ± 0.0547</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Safety factor (SF)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RBF (Gaussian)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>C^inf (Vô hạn lần khả vi, nguy cơ quá trơn làm mờ đỉnh ứng suất)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.9969</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.2419</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1584</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.1138</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5.874</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>-0.8108 ± 0.9292</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.148 ± 0.0547</t>
         </is>
       </c>
     </row>

</xml_diff>